<commit_message>
More icons, track failure interface
</commit_message>
<xml_diff>
--- a/TrackModel/Blue Line.xlsx
+++ b/TrackModel/Blue Line.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pitt-my.sharepoint.com/personal/dgs44_pitt_edu/Documents/Trains/TrackModel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="109" documentId="8_{D0660D75-C052-4898-8402-12AA78E71664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B6A359F-B8BD-4A07-AAFC-47B992CE1F65}"/>
+  <xr:revisionPtr revIDLastSave="129" documentId="8_{D0660D75-C052-4898-8402-12AA78E71664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8DF945D-FFB1-4EE8-82A2-E876714E4517}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C71A2FFE-490E-4D57-BAA4-DE7AC575C897}"/>
+    <workbookView xWindow="6240" yWindow="2430" windowWidth="13125" windowHeight="11295" xr2:uid="{C71A2FFE-490E-4D57-BAA4-DE7AC575C897}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="31">
   <si>
     <t>Blue</t>
   </si>
@@ -114,6 +114,21 @@
   </si>
   <si>
     <t>Y2</t>
+  </si>
+  <si>
+    <t>Station B</t>
+  </si>
+  <si>
+    <t>Station C</t>
+  </si>
+  <si>
+    <t>Block 12</t>
+  </si>
+  <si>
+    <t>Block 6</t>
+  </si>
+  <si>
+    <t>Block 5</t>
   </si>
 </sst>
 </file>
@@ -512,7 +527,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13190075-78CA-4D81-A78A-8327AF8C2968}">
-  <dimension ref="A1:S18"/>
+  <dimension ref="A1:S19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="11" width="9.140625" style="4"/>
@@ -670,7 +685,7 @@
         <v>18</v>
       </c>
       <c r="P3" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q3" s="4">
         <v>0</v>
@@ -858,7 +873,10 @@
         <v>6</v>
       </c>
       <c r="K8" s="2">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>30</v>
       </c>
       <c r="P8" s="4">
         <v>5</v>
@@ -896,6 +914,9 @@
       <c r="H9" s="4">
         <v>0</v>
       </c>
+      <c r="L9" s="4" t="s">
+        <v>29</v>
+      </c>
       <c r="P9" s="4">
         <v>6</v>
       </c>
@@ -1005,7 +1026,7 @@
         <v>0</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="P12" s="4">
         <v>9</v>
@@ -1063,39 +1084,38 @@
       </c>
     </row>
     <row r="14" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>3</v>
+      <c r="A14" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>2</v>
       </c>
       <c r="C14" s="2">
         <v>11</v>
       </c>
-      <c r="D14" s="2">
-        <v>50</v>
-      </c>
-      <c r="E14" s="2">
-        <v>0</v>
-      </c>
-      <c r="F14" s="2">
-        <v>50</v>
-      </c>
-      <c r="G14" s="2"/>
+      <c r="D14" s="4">
+        <v>50</v>
+      </c>
+      <c r="E14" s="4">
+        <v>0</v>
+      </c>
+      <c r="F14" s="4">
+        <v>50</v>
+      </c>
       <c r="H14" s="4">
         <v>0</v>
       </c>
       <c r="P14" s="4">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="Q14" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R14" s="4">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="S14" s="4">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
@@ -1121,14 +1141,17 @@
       <c r="H15" s="4">
         <v>0</v>
       </c>
+      <c r="L15" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="P15" s="4">
+        <v>6</v>
+      </c>
+      <c r="Q15" s="4">
+        <v>0</v>
+      </c>
+      <c r="R15" s="4">
         <v>7</v>
-      </c>
-      <c r="Q15" s="4">
-        <v>-1</v>
-      </c>
-      <c r="R15" s="4">
-        <v>8</v>
       </c>
       <c r="S15" s="4">
         <v>-1</v>
@@ -1158,13 +1181,13 @@
         <v>0</v>
       </c>
       <c r="P16" s="4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q16" s="4">
         <v>-1</v>
       </c>
       <c r="R16" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S16" s="4">
         <v>-1</v>
@@ -1193,17 +1216,14 @@
       <c r="H17" s="4">
         <v>0</v>
       </c>
-      <c r="L17" s="4" t="s">
-        <v>4</v>
-      </c>
       <c r="P17" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q17" s="4">
         <v>-1</v>
       </c>
       <c r="R17" s="4">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="S17" s="4">
         <v>-1</v>
@@ -1232,22 +1252,61 @@
       <c r="H18" s="4">
         <v>0</v>
       </c>
-      <c r="M18" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="N18" s="4" t="s">
-        <v>18</v>
+      <c r="L18" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="P18" s="4">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q18" s="4">
         <v>-1</v>
       </c>
       <c r="R18" s="4">
+        <v>10</v>
+      </c>
+      <c r="S18" s="4">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19" s="4">
+        <v>16</v>
+      </c>
+      <c r="D19" s="2">
+        <v>50</v>
+      </c>
+      <c r="E19" s="2">
+        <v>0</v>
+      </c>
+      <c r="F19" s="2">
+        <v>50</v>
+      </c>
+      <c r="G19" s="2"/>
+      <c r="H19" s="4">
+        <v>0</v>
+      </c>
+      <c r="M19" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="N19" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="P19" s="4">
+        <v>10</v>
+      </c>
+      <c r="Q19" s="4">
+        <v>-1</v>
+      </c>
+      <c r="R19" s="4">
         <v>11</v>
       </c>
-      <c r="S18" s="4">
+      <c r="S19" s="4">
         <v>-1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Green line, changing icon sizes
</commit_message>
<xml_diff>
--- a/TrackModel/Blue Line.xlsx
+++ b/TrackModel/Blue Line.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pitt-my.sharepoint.com/personal/dgs44_pitt_edu/Documents/Trains/TrackModel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="129" documentId="8_{D0660D75-C052-4898-8402-12AA78E71664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8DF945D-FFB1-4EE8-82A2-E876714E4517}"/>
+  <xr:revisionPtr revIDLastSave="130" documentId="8_{D0660D75-C052-4898-8402-12AA78E71664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A1C5A59-1331-4037-B692-EB2006869A7E}"/>
   <bookViews>
-    <workbookView xWindow="6240" yWindow="2430" windowWidth="13125" windowHeight="11295" xr2:uid="{C71A2FFE-490E-4D57-BAA4-DE7AC575C897}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C71A2FFE-490E-4D57-BAA4-DE7AC575C897}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1025,9 +1025,6 @@
       <c r="H12" s="4">
         <v>0</v>
       </c>
-      <c r="L12" s="4" t="s">
-        <v>26</v>
-      </c>
       <c r="P12" s="4">
         <v>9</v>
       </c>
@@ -1064,11 +1061,8 @@
       <c r="H13" s="4">
         <v>0</v>
       </c>
-      <c r="M13" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="N13" s="4" t="s">
-        <v>18</v>
+      <c r="L13" s="4" t="s">
+        <v>26</v>
       </c>
       <c r="P13" s="4">
         <v>10</v>
@@ -1104,6 +1098,12 @@
       </c>
       <c r="H14" s="4">
         <v>0</v>
+      </c>
+      <c r="M14" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="N14" s="4" t="s">
+        <v>18</v>
       </c>
       <c r="P14" s="4">
         <v>11</v>

</xml_diff>